<commit_message>
feat(data): nouvelle liste joueurs Groupe A et B
</commit_message>
<xml_diff>
--- a/public/data/@Liste GROUPE B.xlsx
+++ b/public/data/@Liste GROUPE B.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="555">
   <si>
     <t xml:space="preserve">Équipe </t>
   </si>
@@ -401,10 +401,10 @@
     <t>2XL</t>
   </si>
   <si>
-    <t>DAVID ALEXANDRE</t>
-  </si>
-  <si>
-    <t>SIMOES</t>
+    <t xml:space="preserve">MULLER </t>
+  </si>
+  <si>
+    <t>TITINGUERA</t>
   </si>
   <si>
     <t>LÉO EMILIEN</t>
@@ -1544,10 +1544,7 @@
     <t>VÉRON</t>
   </si>
   <si>
-    <t>FAHMAN</t>
-  </si>
-  <si>
-    <t>GUIRO</t>
+    <t>MANA</t>
   </si>
   <si>
     <t>NOM DE L'ÉQUIPE :GUINÉE 🇬🇳</t>
@@ -2030,7 +2027,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="125">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2349,6 +2346,9 @@
     <xf borderId="1" fillId="3" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
@@ -2902,7 +2902,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -2925,7 +2925,7 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -2937,7 +2937,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -2949,7 +2949,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -2961,7 +2961,7 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -3048,13 +3048,13 @@
         <v>184</v>
       </c>
       <c r="E8" s="73" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F8" s="40">
         <v>26.0</v>
       </c>
       <c r="G8" s="41" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H8" s="28"/>
       <c r="I8" s="29"/>
@@ -3084,13 +3084,13 @@
         <v>141</v>
       </c>
       <c r="E9" s="73" t="s">
+        <v>510</v>
+      </c>
+      <c r="F9" s="117">
+        <v>22.0</v>
+      </c>
+      <c r="G9" s="118" t="s">
         <v>511</v>
-      </c>
-      <c r="F9" s="116">
-        <v>22.0</v>
-      </c>
-      <c r="G9" s="117" t="s">
-        <v>512</v>
       </c>
       <c r="H9" s="31"/>
       <c r="I9" s="32"/>
@@ -3117,16 +3117,16 @@
         <v>76</v>
       </c>
       <c r="D10" s="73" t="s">
+        <v>512</v>
+      </c>
+      <c r="E10" s="73" t="s">
         <v>513</v>
       </c>
-      <c r="E10" s="73" t="s">
+      <c r="F10" s="117">
+        <v>30.0</v>
+      </c>
+      <c r="G10" s="118" t="s">
         <v>514</v>
-      </c>
-      <c r="F10" s="116">
-        <v>30.0</v>
-      </c>
-      <c r="G10" s="117" t="s">
-        <v>515</v>
       </c>
       <c r="H10" s="28"/>
       <c r="I10" s="29"/>
@@ -3149,20 +3149,20 @@
       <c r="B11" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C11" s="117" t="s">
+      <c r="C11" s="118" t="s">
         <v>76</v>
       </c>
       <c r="D11" s="73" t="s">
+        <v>515</v>
+      </c>
+      <c r="E11" s="73" t="s">
         <v>516</v>
       </c>
-      <c r="E11" s="73" t="s">
+      <c r="F11" s="117">
+        <v>25.0</v>
+      </c>
+      <c r="G11" s="118" t="s">
         <v>517</v>
-      </c>
-      <c r="F11" s="116">
-        <v>25.0</v>
-      </c>
-      <c r="G11" s="117" t="s">
-        <v>518</v>
       </c>
       <c r="H11" s="28"/>
       <c r="I11" s="29"/>
@@ -3185,18 +3185,18 @@
       <c r="B12" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="117" t="s">
+      <c r="C12" s="118" t="s">
         <v>76</v>
       </c>
       <c r="D12" s="73" t="s">
+        <v>518</v>
+      </c>
+      <c r="E12" s="73" t="s">
         <v>519</v>
-      </c>
-      <c r="E12" s="73" t="s">
-        <v>520</v>
       </c>
       <c r="F12" s="40"/>
       <c r="G12" s="41" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H12" s="28"/>
       <c r="I12" s="29"/>
@@ -3219,20 +3219,20 @@
       <c r="B13" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="117" t="s">
+      <c r="C13" s="118" t="s">
         <v>86</v>
       </c>
       <c r="D13" s="73" t="s">
         <v>394</v>
       </c>
       <c r="E13" s="73" t="s">
+        <v>521</v>
+      </c>
+      <c r="F13" s="117">
+        <v>25.0</v>
+      </c>
+      <c r="G13" s="118" t="s">
         <v>522</v>
-      </c>
-      <c r="F13" s="116">
-        <v>25.0</v>
-      </c>
-      <c r="G13" s="117" t="s">
-        <v>523</v>
       </c>
       <c r="H13" s="28"/>
       <c r="I13" s="29"/>
@@ -3255,20 +3255,20 @@
       <c r="B14" s="73" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="117" t="s">
+      <c r="C14" s="118" t="s">
         <v>94</v>
       </c>
       <c r="D14" s="73" t="s">
         <v>394</v>
       </c>
       <c r="E14" s="73" t="s">
-        <v>524</v>
-      </c>
-      <c r="F14" s="116">
+        <v>523</v>
+      </c>
+      <c r="F14" s="117">
         <v>30.0</v>
       </c>
-      <c r="G14" s="117" t="s">
-        <v>523</v>
+      <c r="G14" s="118" t="s">
+        <v>522</v>
       </c>
       <c r="H14" s="28"/>
       <c r="I14" s="29"/>
@@ -3295,16 +3295,16 @@
         <v>86</v>
       </c>
       <c r="D15" s="73" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E15" s="73" t="s">
+        <v>521</v>
+      </c>
+      <c r="F15" s="117">
+        <v>22.0</v>
+      </c>
+      <c r="G15" s="118" t="s">
         <v>522</v>
-      </c>
-      <c r="F15" s="116">
-        <v>22.0</v>
-      </c>
-      <c r="G15" s="117" t="s">
-        <v>523</v>
       </c>
       <c r="H15" s="28"/>
       <c r="I15" s="29"/>
@@ -3334,11 +3334,11 @@
         <v>363</v>
       </c>
       <c r="E16" s="73" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="F16" s="40"/>
       <c r="G16" s="41" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H16" s="28"/>
       <c r="I16" s="29"/>
@@ -3361,20 +3361,20 @@
       <c r="B17" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="C17" s="117" t="s">
+      <c r="C17" s="118" t="s">
         <v>86</v>
       </c>
       <c r="D17" s="73" t="s">
+        <v>527</v>
+      </c>
+      <c r="E17" s="73" t="s">
         <v>528</v>
       </c>
-      <c r="E17" s="73" t="s">
-        <v>529</v>
-      </c>
-      <c r="F17" s="116">
+      <c r="F17" s="117">
         <v>27.0</v>
       </c>
-      <c r="G17" s="117" t="s">
-        <v>515</v>
+      <c r="G17" s="118" t="s">
+        <v>514</v>
       </c>
       <c r="H17" s="31"/>
       <c r="I17" s="32"/>
@@ -3397,20 +3397,20 @@
       <c r="B18" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="117" t="s">
+      <c r="C18" s="118" t="s">
         <v>94</v>
       </c>
       <c r="D18" s="73" t="s">
+        <v>529</v>
+      </c>
+      <c r="E18" s="73" t="s">
         <v>530</v>
       </c>
-      <c r="E18" s="73" t="s">
-        <v>531</v>
-      </c>
-      <c r="F18" s="116">
+      <c r="F18" s="117">
         <v>23.0</v>
       </c>
-      <c r="G18" s="117" t="s">
-        <v>523</v>
+      <c r="G18" s="118" t="s">
+        <v>522</v>
       </c>
       <c r="H18" s="28"/>
       <c r="I18" s="29"/>
@@ -3433,20 +3433,20 @@
       <c r="B19" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="117" t="s">
+      <c r="C19" s="118" t="s">
         <v>76</v>
       </c>
       <c r="D19" s="73" t="s">
         <v>179</v>
       </c>
       <c r="E19" s="73" t="s">
-        <v>532</v>
-      </c>
-      <c r="F19" s="116">
+        <v>531</v>
+      </c>
+      <c r="F19" s="117">
         <v>30.0</v>
       </c>
-      <c r="G19" s="117" t="s">
-        <v>515</v>
+      <c r="G19" s="118" t="s">
+        <v>514</v>
       </c>
       <c r="H19" s="31"/>
       <c r="I19" s="32"/>
@@ -3469,18 +3469,18 @@
       <c r="B20" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="117" t="s">
+      <c r="C20" s="118" t="s">
         <v>86</v>
       </c>
       <c r="D20" s="73" t="s">
+        <v>532</v>
+      </c>
+      <c r="E20" s="73" t="s">
         <v>533</v>
       </c>
-      <c r="E20" s="73" t="s">
-        <v>534</v>
-      </c>
       <c r="F20" s="3"/>
-      <c r="G20" s="117" t="s">
-        <v>523</v>
+      <c r="G20" s="118" t="s">
+        <v>522</v>
       </c>
       <c r="H20" s="31"/>
       <c r="I20" s="32"/>
@@ -3503,20 +3503,20 @@
       <c r="B21" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C21" s="117" t="s">
+      <c r="C21" s="118" t="s">
         <v>94</v>
       </c>
       <c r="D21" s="73" t="s">
+        <v>534</v>
+      </c>
+      <c r="E21" s="73" t="s">
         <v>535</v>
       </c>
-      <c r="E21" s="73" t="s">
-        <v>536</v>
-      </c>
-      <c r="F21" s="116">
+      <c r="F21" s="117">
         <v>18.0</v>
       </c>
-      <c r="G21" s="117" t="s">
-        <v>521</v>
+      <c r="G21" s="118" t="s">
+        <v>520</v>
       </c>
       <c r="H21" s="31"/>
       <c r="I21" s="32"/>
@@ -3536,7 +3536,7 @@
       <c r="A22" s="72">
         <v>15.0</v>
       </c>
-      <c r="B22" s="118" t="s">
+      <c r="B22" s="119" t="s">
         <v>102</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -3546,13 +3546,13 @@
         <v>363</v>
       </c>
       <c r="E22" s="73" t="s">
-        <v>537</v>
-      </c>
-      <c r="F22" s="116">
+        <v>536</v>
+      </c>
+      <c r="F22" s="117">
         <v>23.0</v>
       </c>
-      <c r="G22" s="117" t="s">
-        <v>523</v>
+      <c r="G22" s="118" t="s">
+        <v>522</v>
       </c>
       <c r="H22" s="28"/>
       <c r="I22" s="29"/>
@@ -3572,23 +3572,23 @@
       <c r="A23" s="74">
         <v>16.0</v>
       </c>
-      <c r="B23" s="118" t="s">
+      <c r="B23" s="119" t="s">
         <v>102</v>
       </c>
-      <c r="C23" s="117" t="s">
+      <c r="C23" s="118" t="s">
         <v>86</v>
       </c>
       <c r="D23" s="73" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="E23" s="73" t="s">
-        <v>514</v>
-      </c>
-      <c r="F23" s="116">
+        <v>513</v>
+      </c>
+      <c r="F23" s="117">
         <v>22.0</v>
       </c>
-      <c r="G23" s="117" t="s">
-        <v>523</v>
+      <c r="G23" s="118" t="s">
+        <v>522</v>
       </c>
       <c r="H23" s="31"/>
       <c r="I23" s="32"/>
@@ -3605,26 +3605,26 @@
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="119">
+      <c r="A24" s="120">
         <v>17.0</v>
       </c>
-      <c r="B24" s="120" t="s">
+      <c r="B24" s="121" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="121" t="s">
+      <c r="C24" s="122" t="s">
         <v>94</v>
       </c>
       <c r="D24" s="82" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E24" s="82" t="s">
         <v>185</v>
       </c>
-      <c r="F24" s="116">
+      <c r="F24" s="117">
         <v>30.0</v>
       </c>
-      <c r="G24" s="117" t="s">
-        <v>515</v>
+      <c r="G24" s="118" t="s">
+        <v>514</v>
       </c>
       <c r="H24" s="28"/>
       <c r="I24" s="29"/>
@@ -3647,20 +3647,20 @@
       <c r="B25" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="C25" s="117" t="s">
+      <c r="C25" s="118" t="s">
         <v>94</v>
       </c>
       <c r="D25" s="73" t="s">
         <v>358</v>
       </c>
       <c r="E25" s="73" t="s">
-        <v>540</v>
-      </c>
-      <c r="F25" s="116">
+        <v>539</v>
+      </c>
+      <c r="F25" s="117">
         <v>19.0</v>
       </c>
-      <c r="G25" s="117" t="s">
-        <v>523</v>
+      <c r="G25" s="118" t="s">
+        <v>522</v>
       </c>
       <c r="H25" s="28"/>
       <c r="I25" s="29"/>
@@ -3683,18 +3683,18 @@
       <c r="B26" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="117" t="s">
+      <c r="C26" s="118" t="s">
         <v>94</v>
       </c>
       <c r="D26" s="73" t="s">
+        <v>540</v>
+      </c>
+      <c r="E26" s="73" t="s">
         <v>541</v>
-      </c>
-      <c r="E26" s="73" t="s">
-        <v>542</v>
       </c>
       <c r="F26" s="40"/>
       <c r="G26" s="41" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H26" s="31"/>
       <c r="I26" s="32"/>
@@ -3717,20 +3717,20 @@
       <c r="B27" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="117" t="s">
+      <c r="C27" s="118" t="s">
         <v>86</v>
       </c>
       <c r="D27" s="73" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="E27" s="73" t="s">
         <v>185</v>
       </c>
-      <c r="F27" s="116">
+      <c r="F27" s="117">
         <v>22.0</v>
       </c>
-      <c r="G27" s="117" t="s">
-        <v>521</v>
+      <c r="G27" s="118" t="s">
+        <v>520</v>
       </c>
       <c r="H27" s="31"/>
       <c r="I27" s="32"/>
@@ -3747,26 +3747,26 @@
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="119">
+      <c r="A28" s="120">
         <v>21.0</v>
       </c>
-      <c r="B28" s="120" t="s">
+      <c r="B28" s="121" t="s">
         <v>67</v>
       </c>
-      <c r="C28" s="121" t="s">
+      <c r="C28" s="122" t="s">
         <v>94</v>
       </c>
       <c r="D28" s="82" t="s">
+        <v>543</v>
+      </c>
+      <c r="E28" s="82" t="s">
         <v>544</v>
-      </c>
-      <c r="E28" s="82" t="s">
-        <v>545</v>
       </c>
       <c r="F28" s="102">
         <v>23.0</v>
       </c>
       <c r="G28" s="103" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H28" s="64"/>
       <c r="I28" s="65"/>
@@ -3793,16 +3793,16 @@
         <v>76</v>
       </c>
       <c r="D29" s="73" t="s">
+        <v>545</v>
+      </c>
+      <c r="E29" s="73" t="s">
         <v>546</v>
-      </c>
-      <c r="E29" s="73" t="s">
-        <v>547</v>
       </c>
       <c r="F29" s="40">
         <v>22.0</v>
       </c>
       <c r="G29" s="41" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H29" s="31"/>
       <c r="I29" s="32"/>
@@ -3825,20 +3825,20 @@
       <c r="B30" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C30" s="117" t="s">
+      <c r="C30" s="118" t="s">
         <v>86</v>
       </c>
       <c r="D30" s="73" t="s">
+        <v>547</v>
+      </c>
+      <c r="E30" s="73" t="s">
         <v>548</v>
       </c>
-      <c r="E30" s="73" t="s">
+      <c r="F30" s="117">
+        <v>21.0</v>
+      </c>
+      <c r="G30" s="118" t="s">
         <v>549</v>
-      </c>
-      <c r="F30" s="116">
-        <v>21.0</v>
-      </c>
-      <c r="G30" s="117" t="s">
-        <v>550</v>
       </c>
       <c r="H30" s="31"/>
       <c r="I30" s="32"/>
@@ -3865,16 +3865,16 @@
         <v>76</v>
       </c>
       <c r="D31" s="73" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="E31" s="73" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F31" s="40">
         <v>30.0</v>
       </c>
       <c r="G31" s="41" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H31" s="31"/>
       <c r="I31" s="32"/>
@@ -3897,20 +3897,20 @@
       <c r="B32" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="117" t="s">
+      <c r="C32" s="118" t="s">
         <v>76</v>
       </c>
       <c r="D32" s="73" t="s">
+        <v>551</v>
+      </c>
+      <c r="E32" s="73" t="s">
         <v>552</v>
       </c>
-      <c r="E32" s="73" t="s">
+      <c r="F32" s="123">
+        <v>23.0</v>
+      </c>
+      <c r="G32" s="124" t="s">
         <v>553</v>
-      </c>
-      <c r="F32" s="122">
-        <v>23.0</v>
-      </c>
-      <c r="G32" s="123" t="s">
-        <v>554</v>
       </c>
       <c r="H32" s="64"/>
       <c r="I32" s="65"/>
@@ -3937,14 +3937,14 @@
         <v>94</v>
       </c>
       <c r="D33" s="73" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="E33" s="73" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F33" s="3"/>
-      <c r="G33" s="117" t="s">
-        <v>521</v>
+      <c r="G33" s="118" t="s">
+        <v>520</v>
       </c>
       <c r="H33" s="31"/>
       <c r="I33" s="32"/>
@@ -12616,11 +12616,11 @@
       <c r="C33" s="111" t="s">
         <v>76</v>
       </c>
-      <c r="D33" s="112" t="s">
+      <c r="D33" s="116" t="s">
+        <v>181</v>
+      </c>
+      <c r="E33" s="116" t="s">
         <v>502</v>
-      </c>
-      <c r="E33" s="112" t="s">
-        <v>503</v>
       </c>
       <c r="F33" s="40"/>
       <c r="G33" s="41"/>

</xml_diff>